<commit_message>
Refactor and update result files and scripts - Updated multiple result files (newfile5th4.txt, newfile5th5.txt, newfile6th3.txt, newfile6th4.txt, newfile7th3.txt, newfile7th4.txt, newfile8th3.txt, newfile9th3.txt) to modify the data format and structure. - Changed the way results are appended in the script `02_split_results_to_pXsY.py` for better clarity and consistency. - Introduced a new script `01_generate_table1.py` to generate a summary table from the union gene results, including support counts for different periods.
</commit_message>
<xml_diff>
--- a/results/components/gene_names/p10s3.xlsx
+++ b/results/components/gene_names/p10s3.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>gene1</t>
   </si>
@@ -22,16 +22,34 @@
     <t>gene2</t>
   </si>
   <si>
-    <t>Psn</t>
-  </si>
-  <si>
-    <t>Ark</t>
-  </si>
-  <si>
-    <t>bib</t>
-  </si>
-  <si>
-    <t>noc</t>
+    <t>Ef1gamma</t>
+  </si>
+  <si>
+    <t>tin</t>
+  </si>
+  <si>
+    <t>Mmp1</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>Dif</t>
+  </si>
+  <si>
+    <t>Rca1</t>
+  </si>
+  <si>
+    <t>sgg</t>
+  </si>
+  <si>
+    <t>pot</t>
+  </si>
+  <si>
+    <t>cactin</t>
+  </si>
+  <si>
+    <t>PebIII</t>
   </si>
 </sst>
 </file>
@@ -363,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -390,6 +408,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
recent attempts of reproducing tables
</commit_message>
<xml_diff>
--- a/results/components/gene_names/p10s3.xlsx
+++ b/results/components/gene_names/p10s3.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
   <si>
     <t>gene1</t>
   </si>
@@ -22,34 +22,103 @@
     <t>gene2</t>
   </si>
   <si>
-    <t>Ef1gamma</t>
-  </si>
-  <si>
-    <t>tin</t>
-  </si>
-  <si>
-    <t>Mmp1</t>
-  </si>
-  <si>
-    <t>v</t>
-  </si>
-  <si>
-    <t>Dif</t>
-  </si>
-  <si>
-    <t>Rca1</t>
-  </si>
-  <si>
-    <t>sgg</t>
-  </si>
-  <si>
-    <t>pot</t>
-  </si>
-  <si>
-    <t>cactin</t>
-  </si>
-  <si>
-    <t>PebIII</t>
+    <t>Syx1A</t>
+  </si>
+  <si>
+    <t>CG32082</t>
+  </si>
+  <si>
+    <t>eve</t>
+  </si>
+  <si>
+    <t>CG13850</t>
+  </si>
+  <si>
+    <t>Sxl</t>
+  </si>
+  <si>
+    <t>gl</t>
+  </si>
+  <si>
+    <t>oaf</t>
+  </si>
+  <si>
+    <t>Akap200</t>
+  </si>
+  <si>
+    <t>Mef2</t>
+  </si>
+  <si>
+    <t>shot</t>
+  </si>
+  <si>
+    <t>Apc</t>
+  </si>
+  <si>
+    <t>caps</t>
+  </si>
+  <si>
+    <t>CG16719</t>
+  </si>
+  <si>
+    <t>rdo</t>
+  </si>
+  <si>
+    <t>tral</t>
+  </si>
+  <si>
+    <t>esc</t>
+  </si>
+  <si>
+    <t>dmt</t>
+  </si>
+  <si>
+    <t>stumps</t>
+  </si>
+  <si>
+    <t>Sin3A</t>
+  </si>
+  <si>
+    <t>Nrt</t>
+  </si>
+  <si>
+    <t>Hs6st</t>
+  </si>
+  <si>
+    <t>Snap</t>
+  </si>
+  <si>
+    <t>Hmgs</t>
+  </si>
+  <si>
+    <t>betaTub56D</t>
+  </si>
+  <si>
+    <t>Caf1</t>
+  </si>
+  <si>
+    <t>Idgf4</t>
+  </si>
+  <si>
+    <t>CG17739</t>
+  </si>
+  <si>
+    <t>Ddx1</t>
+  </si>
+  <si>
+    <t>sav</t>
+  </si>
+  <si>
+    <t>crol</t>
+  </si>
+  <si>
+    <t>ry</t>
+  </si>
+  <si>
+    <t>Sur</t>
+  </si>
+  <si>
+    <t>acj6</t>
   </si>
 </sst>
 </file>
@@ -381,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -432,6 +501,110 @@
         <v>11</v>
       </c>
     </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>